<commit_message>
datos: actualizacion automatica 2026-08-07 01:50 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1,30 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PORTADA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RANKING" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESCALAS DE TASA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIMULADOR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASA BCRP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="PORTADA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RANKING" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ESCALAS DE TASA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SIMULADOR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TASA BCRP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -237,9 +235,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -357,13 +352,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -387,7 +382,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -439,13 +434,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -469,7 +464,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -518,13 +513,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -547,14 +542,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -594,8 +589,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -621,7 +616,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>15</col>
@@ -636,9 +631,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -648,7 +643,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -663,9 +658,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -675,7 +670,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -690,9 +685,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1011,7 +1006,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1081,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 06/08/2026 15:42. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 07/08/2026 01:50. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1323,873 +1318,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 06/08/2026 15:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Entidad/tema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de fuente</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F28"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2229,7 +1357,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -3411,7 +2539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -4226,7 +3354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -4828,7 +3956,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -5386,7 +4514,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5104,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -7043,7 +6171,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
@@ -7819,635 +6947,863 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 06/08/2026 15:42</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 01:50</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de entidad</t>
+          <t>Entidad/tema</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo de fuente</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Analizada en el portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Banco de Crédito del Perú</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Interbank</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Citibank del Perú</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Scotiabank Perú</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>BBVA</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Bancom</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Banco Pichincha</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>BANBIF</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Mibanco</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Banco Falabella</t>
         </is>
       </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Banco Ripley</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Alfin Banco</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Banco Santander</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Banco GNB</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>ICBC Peru bank</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Bank of China(Perú)</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Banco BCI</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Compartamos Banco</t>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Banco Efectiva</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
         </is>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Proempresa</t>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>InFinance XP</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Surgir</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Arequipa</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Cuzco</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Huancayo</t>
-        </is>
-      </c>
-      <c r="C32" s="30" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Ica</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B34" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Maynas</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Del Santa</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Paita</t>
-        </is>
-      </c>
-      <c r="C36" s="30" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Piura</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Tacna</t>
-        </is>
-      </c>
-      <c r="C38" s="30" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Trujillo</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Caja Metropolitana</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Los Andes</t>
-        </is>
-      </c>
-      <c r="C41" s="30" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Prymera</t>
-        </is>
-      </c>
-      <c r="C42" s="30" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Incasur</t>
-        </is>
-      </c>
-      <c r="C43" s="30" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Del Centro</t>
-        </is>
-      </c>
-      <c r="C44" s="30" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Cencosud Scotia</t>
-        </is>
-      </c>
-      <c r="C45" s="30" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C45"/>
+  <autoFilter ref="A4:F28"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-07 02:31 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,14 +15,16 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -235,6 +237,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1006,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 07/08/2026 01:50. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 07/08/2026 02:31. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1323,873 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 02:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Entidad/tema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de fuente</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F28"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1357,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -3354,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -3956,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -4514,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -6171,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
@@ -6947,863 +7819,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 01:50</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 02:31</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Entidad/tema</t>
+          <t>Tipo de entidad</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de fuente</t>
+          <t>Entidad</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
+          <t>Analizada en el portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Interbank</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Citibank del Perú</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Bancom</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Banco Pichincha</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>BANBIF</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Mibanco</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Alfin Banco</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Banco Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Banco GNB</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ICBC Peru bank</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Bank of China(Perú)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Banco BCI</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Compartamos Banco</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Banco Efectiva</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Financiera QAPAQ</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Proempresa</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>InFinance XP</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Surgir</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Arequipa</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Cuzco</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Huancayo</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Ica</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Maynas</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Del Santa</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Paita</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Piura</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Tacna</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Trujillo</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>Caja Metropolitana</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Los Andes</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Prymera</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Incasur</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Del Centro</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Cencosud Scotia</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="inlineStr">
+        <is>
+          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F28"/>
+  <autoFilter ref="A4:C45"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-07 03:26 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 07/08/2026 02:31. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 07/08/2026 03:26. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 02:31</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 03:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-07 11:43 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 07/08/2026 03:26. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 07/08/2026 11:43. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 03:26</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 11:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-07 23:30 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 07/08/2026 11:43. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 07/08/2026 23:30. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 11:43</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 23:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-08 11:25 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 07/08/2026 23:30. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 08/08/2026 11:25. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 07/08/2026 23:30</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 08/08/2026 11:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-08 23:25 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 08/08/2026 11:25. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 08/08/2026 23:25. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 08/08/2026 11:25</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 08/08/2026 23:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-09 11:25 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 08/08/2026 23:25. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 09/08/2026 11:25. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 08/08/2026 23:25</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 09/08/2026 11:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-09 23:28 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 09/08/2026 11:25. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 09/08/2026 23:28. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 09/08/2026 11:25</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 09/08/2026 23:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-10 11:44 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 09/08/2026 23:28. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 10/08/2026 11:44. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 09/08/2026 23:28</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 10/08/2026 11:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-10 23:31 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 10/08/2026 11:44. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 10/08/2026 23:31. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 10/08/2026 11:44</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 10/08/2026 23:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-11 11:41 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 10/08/2026 23:31. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 11/08/2026 11:41. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 10/08/2026 23:31</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 11/08/2026 11:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-11 23:36 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 11/08/2026 11:41. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 11/08/2026 23:36. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 11/08/2026 11:41</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 11/08/2026 23:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-12 11:42 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 11/08/2026 23:36. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 12/08/2026 11:42. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 11/08/2026 23:36</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 12/08/2026 11:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-12 23:37 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 12/08/2026 11:42. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 12/08/2026 23:37. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 12/08/2026 11:42</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 12/08/2026 23:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-13 11:43 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 12/08/2026 23:37. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 13/08/2026 11:43. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 12/08/2026 23:37</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 13/08/2026 11:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-13 23:37 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 13/08/2026 11:43. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 13/08/2026 23:37. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 13/08/2026 11:43</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 13/08/2026 23:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-14 11:41 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 13/08/2026 23:37. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 14/08/2026 11:41. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 13/08/2026 23:37</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 14/08/2026 11:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-14 23:18 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 14/08/2026 11:41. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 14/08/2026 23:18. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 14/08/2026 11:41</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 14/08/2026 23:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-15 11:16 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 14/08/2026 23:18. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 15/08/2026 11:16. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 14/08/2026 23:18</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 15/08/2026 11:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-15 23:17 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 15/08/2026 11:16. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 15/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 15/08/2026 11:16</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 15/08/2026 23:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-16 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 15/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 16/08/2026 11:17. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 15/08/2026 23:17</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 16/08/2026 11:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-16 23:16 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 16/08/2026 11:17. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 16/08/2026 23:16. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 16/08/2026 11:17</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 16/08/2026 23:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-17 11:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 16/08/2026 23:16. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 17/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 16/08/2026 23:16</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 17/08/2026 11:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-17 23:20 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 17/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 17/08/2026 23:20. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 17/08/2026 11:22</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 17/08/2026 23:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-18 11:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 17/08/2026 23:20. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 18/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 17/08/2026 23:20</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 18/08/2026 11:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-18 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,16 +15,14 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -237,9 +235,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -561,12 +556,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'TASA BCRP'!$A$5:$A$40</f>
+              <f>'TASA BCRP'!$A$5:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'TASA BCRP'!$B$5:$B$40</f>
+              <f>'TASA BCRP'!$B$5:$B$41</f>
             </numRef>
           </val>
         </ser>
@@ -1011,7 +1006,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1081,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 18/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 18/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1323,873 +1318,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 18/08/2026 11:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Entidad/tema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de fuente</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F28"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2229,7 +1357,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -3411,7 +2539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4226,7 +3354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4810,7 +3938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4828,7 +3956,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5347,6 +4475,20 @@
       </c>
       <c r="C40" s="29">
         <f>(B40-B39)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C41" s="29">
+        <f>(B41-B40)*100</f>
         <v/>
       </c>
     </row>
@@ -5386,7 +4528,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5118,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7043,7 +6185,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7819,635 +6961,863 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 18/08/2026 11:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 18/08/2026 23:19</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de entidad</t>
+          <t>Entidad/tema</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo de fuente</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Analizada en el portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Banco de Crédito del Perú</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Interbank</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Citibank del Perú</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Scotiabank Perú</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>BBVA</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Bancom</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Banco Pichincha</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>BANBIF</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Mibanco</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Banco Falabella</t>
         </is>
       </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Banco Ripley</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Alfin Banco</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Banco Santander</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Banco GNB</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>ICBC Peru bank</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Bank of China(Perú)</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Banco BCI</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Compartamos Banco</t>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Banco Efectiva</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
         </is>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Proempresa</t>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>InFinance XP</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Surgir</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Arequipa</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Cuzco</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Huancayo</t>
-        </is>
-      </c>
-      <c r="C32" s="30" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Ica</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B34" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Maynas</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Del Santa</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Paita</t>
-        </is>
-      </c>
-      <c r="C36" s="30" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Piura</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Tacna</t>
-        </is>
-      </c>
-      <c r="C38" s="30" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Trujillo</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Caja Metropolitana</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Los Andes</t>
-        </is>
-      </c>
-      <c r="C41" s="30" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Prymera</t>
-        </is>
-      </c>
-      <c r="C42" s="30" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Incasur</t>
-        </is>
-      </c>
-      <c r="C43" s="30" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Del Centro</t>
-        </is>
-      </c>
-      <c r="C44" s="30" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Cencosud Scotia</t>
-        </is>
-      </c>
-      <c r="C45" s="30" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C45"/>
+  <autoFilter ref="A4:F28"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-19 11:21 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,14 +15,16 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -235,6 +237,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1006,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 18/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 19/08/2026 11:21. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1323,873 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 19/08/2026 11:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Entidad/tema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de fuente</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F28"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1357,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -3354,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -3956,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -4528,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -6185,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
@@ -6961,863 +7833,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 18/08/2026 23:19</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 19/08/2026 11:21</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Entidad/tema</t>
+          <t>Tipo de entidad</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de fuente</t>
+          <t>Entidad</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
+          <t>Analizada en el portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Interbank</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Citibank del Perú</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Bancom</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Banco Pichincha</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>BANBIF</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Mibanco</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Alfin Banco</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Banco Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Banco GNB</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ICBC Peru bank</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Bank of China(Perú)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Banco BCI</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Compartamos Banco</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Banco Efectiva</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Financiera QAPAQ</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Proempresa</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>InFinance XP</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Surgir</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Arequipa</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Cuzco</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Huancayo</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Ica</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Maynas</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Del Santa</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Paita</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Piura</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Tacna</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Trujillo</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>Caja Metropolitana</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Los Andes</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Prymera</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Incasur</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Del Centro</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Cencosud Scotia</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="inlineStr">
+        <is>
+          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F28"/>
+  <autoFilter ref="A4:C45"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-19 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 19/08/2026 11:21. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 19/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 19/08/2026 11:21</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 19/08/2026 23:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-20 11:23 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 19/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 20/08/2026 11:23. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 19/08/2026 23:19</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 20/08/2026 11:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-20 23:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 20/08/2026 11:23. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 20/08/2026 23:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 20/08/2026 11:23</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 20/08/2026 23:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-21 11:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 20/08/2026 23:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 21/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 20/08/2026 23:22</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 21/08/2026 11:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-21 23:20 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 21/08/2026 11:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 21/08/2026 23:20. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 21/08/2026 11:22</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 21/08/2026 23:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-22 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 21/08/2026 23:20. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 22/08/2026 11:17. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 21/08/2026 23:20</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 22/08/2026 11:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-22 23:17 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,16 +15,14 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -237,9 +235,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1011,7 +1006,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1081,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 22/08/2026 11:17. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 22/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1323,873 +1318,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 22/08/2026 11:17</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Entidad/tema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de fuente</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F28"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2229,7 +1357,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -3411,7 +2539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4226,7 +3354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4828,7 +3956,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5400,7 +4528,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5118,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7057,7 +6185,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7833,635 +6961,863 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 22/08/2026 11:17</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 22/08/2026 23:17</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de entidad</t>
+          <t>Entidad/tema</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo de fuente</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Analizada en el portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Banco de Crédito del Perú</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Interbank</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Citibank del Perú</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Scotiabank Perú</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>BBVA</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Bancom</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Banco Pichincha</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>BANBIF</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Mibanco</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Banco Falabella</t>
         </is>
       </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Banco Ripley</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Alfin Banco</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Banco Santander</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Banco GNB</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>ICBC Peru bank</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Bank of China(Perú)</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Banco BCI</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Compartamos Banco</t>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Banco Efectiva</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
         </is>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Proempresa</t>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>InFinance XP</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Surgir</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Arequipa</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Cuzco</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Huancayo</t>
-        </is>
-      </c>
-      <c r="C32" s="30" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Ica</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B34" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Maynas</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Del Santa</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Paita</t>
-        </is>
-      </c>
-      <c r="C36" s="30" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Piura</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Tacna</t>
-        </is>
-      </c>
-      <c r="C38" s="30" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Trujillo</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Caja Metropolitana</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Los Andes</t>
-        </is>
-      </c>
-      <c r="C41" s="30" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Prymera</t>
-        </is>
-      </c>
-      <c r="C42" s="30" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Incasur</t>
-        </is>
-      </c>
-      <c r="C43" s="30" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Del Centro</t>
-        </is>
-      </c>
-      <c r="C44" s="30" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Cencosud Scotia</t>
-        </is>
-      </c>
-      <c r="C45" s="30" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C45"/>
+  <autoFilter ref="A4:F28"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-23 11:18 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,14 +15,16 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -235,6 +237,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1006,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 22/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 23/08/2026 11:18. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1323,873 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 23/08/2026 11:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Entidad/tema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de fuente</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F28"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1357,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -3354,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -3956,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -4528,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -6185,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
@@ -6961,863 +7833,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 22/08/2026 23:17</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 23/08/2026 11:18</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Entidad/tema</t>
+          <t>Tipo de entidad</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de fuente</t>
+          <t>Entidad</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
+          <t>Analizada en el portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Interbank</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Citibank del Perú</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Bancom</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Banco Pichincha</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>BANBIF</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Mibanco</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Alfin Banco</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Banco Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Banco GNB</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ICBC Peru bank</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Bank of China(Perú)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Banco BCI</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Compartamos Banco</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Banco Efectiva</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Financiera QAPAQ</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Proempresa</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>InFinance XP</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Surgir</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Arequipa</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Cuzco</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Huancayo</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Ica</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Maynas</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Del Santa</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Paita</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Piura</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Tacna</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Trujillo</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>Caja Metropolitana</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Los Andes</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Prymera</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Incasur</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Del Centro</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Cencosud Scotia</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="inlineStr">
+        <is>
+          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F28"/>
+  <autoFilter ref="A4:C45"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-23 23:17 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 23/08/2026 11:18. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 23/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 23/08/2026 11:18</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 23/08/2026 23:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-24 11:24 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 23/08/2026 23:17. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 24/08/2026 11:24. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 23/08/2026 23:17</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 24/08/2026 11:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-24 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 24/08/2026 11:24. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 24/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 24/08/2026 11:24</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 24/08/2026 23:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-25 11:23 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 24/08/2026 23:19. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 25/08/2026 11:23. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 24/08/2026 23:19</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 25/08/2026 11:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-25 23:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 25/08/2026 11:23. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 25/08/2026 23:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 25/08/2026 11:23</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 25/08/2026 23:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-26 11:26 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 25/08/2026 23:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 26/08/2026 11:26. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 25/08/2026 23:22</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 26/08/2026 11:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-27 04:12 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 26/08/2026 11:26. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 27/08/2026 04:12. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 26/08/2026 11:26</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 27/08/2026 04:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-27 20:53 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 27/08/2026 04:12. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 27/08/2026 20:53. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 27/08/2026 04:12</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 27/08/2026 20:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-28 06:45 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,16 +15,14 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -237,9 +235,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1011,7 +1006,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1081,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 27/08/2026 20:53. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 28/08/2026 06:45. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1323,873 +1318,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 27/08/2026 20:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Entidad/tema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de fuente</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F28"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2229,7 +1357,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -3411,7 +2539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -4226,7 +3354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -4828,7 +3956,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -5400,7 +4528,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5118,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -7057,7 +6185,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
@@ -7833,635 +6961,863 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 27/08/2026 20:53</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 28/08/2026 06:45</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de entidad</t>
+          <t>Entidad/tema</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo de fuente</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Analizada en el portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Banco de Crédito del Perú</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Interbank</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Citibank del Perú</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Scotiabank Perú</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>BBVA</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Bancom</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Banco Pichincha</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>BANBIF</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Mibanco</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Banco Falabella</t>
         </is>
       </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Banco Ripley</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Alfin Banco</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Banco Santander</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Banco GNB</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>ICBC Peru bank</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Bank of China(Perú)</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Banco BCI</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Compartamos Banco</t>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Banco Efectiva</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
         </is>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Proempresa</t>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>InFinance XP</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Surgir</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Arequipa</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Cuzco</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Huancayo</t>
-        </is>
-      </c>
-      <c r="C32" s="30" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Ica</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B34" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Maynas</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Del Santa</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Paita</t>
-        </is>
-      </c>
-      <c r="C36" s="30" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Piura</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Tacna</t>
-        </is>
-      </c>
-      <c r="C38" s="30" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Trujillo</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Caja Metropolitana</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Los Andes</t>
-        </is>
-      </c>
-      <c r="C41" s="30" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Prymera</t>
-        </is>
-      </c>
-      <c r="C42" s="30" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Incasur</t>
-        </is>
-      </c>
-      <c r="C43" s="30" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Del Centro</t>
-        </is>
-      </c>
-      <c r="C44" s="30" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Cencosud Scotia</t>
-        </is>
-      </c>
-      <c r="C45" s="30" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C45"/>
+  <autoFilter ref="A4:F28"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-28 21:18 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,14 +15,16 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -235,6 +237,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1006,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 28/08/2026 06:45. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 28/08/2026 21:18. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1323,873 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 28/08/2026 21:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Entidad/tema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de fuente</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F28"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1357,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -3354,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -3956,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -4528,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -6185,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
@@ -6961,863 +7833,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 28/08/2026 06:45</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 28/08/2026 21:18</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Entidad/tema</t>
+          <t>Tipo de entidad</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de fuente</t>
+          <t>Entidad</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
+          <t>Analizada en el portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Interbank</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Citibank del Perú</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Bancom</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Banco Pichincha</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>BANBIF</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Mibanco</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Alfin Banco</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Banco Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Banco GNB</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ICBC Peru bank</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Bank of China(Perú)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Banco BCI</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Compartamos Banco</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Banco Efectiva</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Financiera QAPAQ</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Proempresa</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>InFinance XP</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Surgir</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Arequipa</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Cuzco</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Huancayo</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Ica</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Maynas</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Del Santa</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Paita</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Piura</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Tacna</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Trujillo</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>Caja Metropolitana</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Los Andes</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Prymera</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Incasur</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Del Centro</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Cencosud Scotia</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="inlineStr">
+        <is>
+          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F28"/>
+  <autoFilter ref="A4:C45"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-29 04:00 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 28/08/2026 21:18. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 29/08/2026 04:00. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 28/08/2026 21:18</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 29/08/2026 04:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-29 15:27 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 29/08/2026 04:00. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 29/08/2026 15:27. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 29/08/2026 04:00</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 29/08/2026 15:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-30 01:00 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -561,12 +561,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'TASA BCRP'!$A$5:$A$41</f>
+              <f>'TASA BCRP'!$A$5:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'TASA BCRP'!$B$5:$B$41</f>
+              <f>'TASA BCRP'!$B$5:$B$35</f>
             </numRef>
           </val>
         </ser>
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 29/08/2026 15:27. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 30/08/2026 01:00. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -4852,22 +4852,22 @@
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>0.0775</v>
+        <v>0.065</v>
       </c>
       <c r="C5" s="24" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>0.075</v>
+        <v>0.0625</v>
       </c>
       <c r="C6" s="29">
         <f>(B6-B5)*100</f>
@@ -4877,11 +4877,11 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>0.0725</v>
+        <v>0.0625</v>
       </c>
       <c r="C7" s="29">
         <f>(B7-B6)*100</f>
@@ -4891,11 +4891,11 @@
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="C8" s="29">
         <f>(B8-B7)*100</f>
@@ -4905,11 +4905,11 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>0.0675</v>
+        <v>0.0575</v>
       </c>
       <c r="C9" s="29">
         <f>(B9-B8)*100</f>
@@ -4919,11 +4919,11 @@
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>0.065</v>
+        <v>0.0575</v>
       </c>
       <c r="C10" s="29">
         <f>(B10-B9)*100</f>
@@ -4933,11 +4933,11 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>0.0625</v>
+        <v>0.0575</v>
       </c>
       <c r="C11" s="29">
         <f>(B11-B10)*100</f>
@@ -4947,11 +4947,11 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>0.0625</v>
+        <v>0.055</v>
       </c>
       <c r="C12" s="29">
         <f>(B12-B11)*100</f>
@@ -4961,11 +4961,11 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>0.06</v>
+        <v>0.0525</v>
       </c>
       <c r="C13" s="29">
         <f>(B13-B12)*100</f>
@@ -4975,11 +4975,11 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.0525</v>
       </c>
       <c r="C14" s="29">
         <f>(B14-B13)*100</f>
@@ -4989,11 +4989,11 @@
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.05</v>
       </c>
       <c r="C15" s="29">
         <f>(B15-B14)*100</f>
@@ -5003,11 +5003,11 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.05</v>
       </c>
       <c r="C16" s="29">
         <f>(B16-B15)*100</f>
@@ -5017,11 +5017,11 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
-        <v>0.055</v>
+        <v>0.0475</v>
       </c>
       <c r="C17" s="29">
         <f>(B17-B16)*100</f>
@@ -5031,11 +5031,11 @@
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
-        <v>0.0525</v>
+        <v>0.0475</v>
       </c>
       <c r="C18" s="29">
         <f>(B18-B17)*100</f>
@@ -5045,11 +5045,11 @@
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
-        <v>0.0525</v>
+        <v>0.0475</v>
       </c>
       <c r="C19" s="29">
         <f>(B19-B18)*100</f>
@@ -5059,11 +5059,11 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
-        <v>0.05</v>
+        <v>0.0475</v>
       </c>
       <c r="C20" s="29">
         <f>(B20-B19)*100</f>
@@ -5073,11 +5073,11 @@
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
-        <v>0.05</v>
+        <v>0.045</v>
       </c>
       <c r="C21" s="29">
         <f>(B21-B20)*100</f>
@@ -5087,11 +5087,11 @@
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.045</v>
       </c>
       <c r="C22" s="29">
         <f>(B22-B21)*100</f>
@@ -5101,11 +5101,11 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.045</v>
       </c>
       <c r="C23" s="29">
         <f>(B23-B22)*100</f>
@@ -5115,11 +5115,11 @@
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.045</v>
       </c>
       <c r="C24" s="29">
         <f>(B24-B23)*100</f>
@@ -5129,11 +5129,11 @@
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.0425</v>
       </c>
       <c r="C25" s="29">
         <f>(B25-B24)*100</f>
@@ -5143,11 +5143,11 @@
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0425</v>
       </c>
       <c r="C26" s="29">
         <f>(B26-B25)*100</f>
@@ -5157,11 +5157,11 @@
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0425</v>
       </c>
       <c r="C27" s="29">
         <f>(B27-B26)*100</f>
@@ -5171,11 +5171,11 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0425</v>
       </c>
       <c r="C28" s="29">
         <f>(B28-B27)*100</f>
@@ -5185,11 +5185,11 @@
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0425</v>
       </c>
       <c r="C29" s="29">
         <f>(B29-B28)*100</f>
@@ -5199,7 +5199,7 @@
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -5213,7 +5213,7 @@
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -5227,7 +5227,7 @@
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -5241,7 +5241,7 @@
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -5255,7 +5255,7 @@
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -5269,7 +5269,7 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -5277,90 +5277,6 @@
       </c>
       <c r="C35" s="29">
         <f>(B35-B34)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C36" s="29">
-        <f>(B36-B35)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="24" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B37" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C37" s="29">
-        <f>(B37-B36)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="24" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B38" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C38" s="29">
-        <f>(B38-B37)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C39" s="29">
-        <f>(B39-B38)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B40" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C40" s="29">
-        <f>(B40-B39)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C41" s="29">
-        <f>(B41-B40)*100</f>
         <v/>
       </c>
     </row>
@@ -5400,7 +5316,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5906,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -7057,7 +6973,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7767,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 29/08/2026 15:27</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 30/08/2026 01:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-30 15:09 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 30/08/2026 01:00. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 30/08/2026 15:09. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 30/08/2026 01:00</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 30/08/2026 15:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-31 01:04 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 30/08/2026 15:09. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 31/08/2026 01:04. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 30/08/2026 15:09</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 31/08/2026 01:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-08-31 17:52 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,16 +15,14 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -237,9 +235,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -561,12 +556,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'TASA BCRP'!$A$5:$A$35</f>
+              <f>'TASA BCRP'!$A$5:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'TASA BCRP'!$B$5:$B$35</f>
+              <f>'TASA BCRP'!$B$5:$B$41</f>
             </numRef>
           </val>
         </ser>
@@ -1011,7 +1006,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1081,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 31/08/2026 01:04. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 31/08/2026 17:52. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1323,873 +1318,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 31/08/2026 01:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Entidad/tema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de fuente</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C8" s="31" t="inlineStr">
-        <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:F28"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2229,7 +1357,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -3411,7 +2539,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -4226,7 +3354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -4810,7 +3938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4828,7 +3956,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -4852,22 +3980,22 @@
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>0.065</v>
+        <v>0.0775</v>
       </c>
       <c r="C5" s="24" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>0.0625</v>
+        <v>0.075</v>
       </c>
       <c r="C6" s="29">
         <f>(B6-B5)*100</f>
@@ -4877,11 +4005,11 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>0.0625</v>
+        <v>0.0725</v>
       </c>
       <c r="C7" s="29">
         <f>(B7-B6)*100</f>
@@ -4891,11 +4019,11 @@
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C8" s="29">
         <f>(B8-B7)*100</f>
@@ -4905,11 +4033,11 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.0675</v>
       </c>
       <c r="C9" s="29">
         <f>(B9-B8)*100</f>
@@ -4919,11 +4047,11 @@
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.065</v>
       </c>
       <c r="C10" s="29">
         <f>(B10-B9)*100</f>
@@ -4933,11 +4061,11 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.0625</v>
       </c>
       <c r="C11" s="29">
         <f>(B11-B10)*100</f>
@@ -4947,11 +4075,11 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>0.055</v>
+        <v>0.0625</v>
       </c>
       <c r="C12" s="29">
         <f>(B12-B11)*100</f>
@@ -4961,11 +4089,11 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>0.0525</v>
+        <v>0.06</v>
       </c>
       <c r="C13" s="29">
         <f>(B13-B12)*100</f>
@@ -4975,11 +4103,11 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>0.0525</v>
+        <v>0.0575</v>
       </c>
       <c r="C14" s="29">
         <f>(B14-B13)*100</f>
@@ -4989,11 +4117,11 @@
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
-        <v>0.05</v>
+        <v>0.0575</v>
       </c>
       <c r="C15" s="29">
         <f>(B15-B14)*100</f>
@@ -5003,11 +4131,11 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>0.05</v>
+        <v>0.0575</v>
       </c>
       <c r="C16" s="29">
         <f>(B16-B15)*100</f>
@@ -5017,11 +4145,11 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.055</v>
       </c>
       <c r="C17" s="29">
         <f>(B17-B16)*100</f>
@@ -5031,11 +4159,11 @@
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.0525</v>
       </c>
       <c r="C18" s="29">
         <f>(B18-B17)*100</f>
@@ -5045,11 +4173,11 @@
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.0525</v>
       </c>
       <c r="C19" s="29">
         <f>(B19-B18)*100</f>
@@ -5059,11 +4187,11 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.05</v>
       </c>
       <c r="C20" s="29">
         <f>(B20-B19)*100</f>
@@ -5073,11 +4201,11 @@
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
-        <v>0.045</v>
+        <v>0.05</v>
       </c>
       <c r="C21" s="29">
         <f>(B21-B20)*100</f>
@@ -5087,11 +4215,11 @@
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0475</v>
       </c>
       <c r="C22" s="29">
         <f>(B22-B21)*100</f>
@@ -5101,11 +4229,11 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0475</v>
       </c>
       <c r="C23" s="29">
         <f>(B23-B22)*100</f>
@@ -5115,11 +4243,11 @@
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0475</v>
       </c>
       <c r="C24" s="29">
         <f>(B24-B23)*100</f>
@@ -5129,11 +4257,11 @@
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
-        <v>0.0425</v>
+        <v>0.0475</v>
       </c>
       <c r="C25" s="29">
         <f>(B25-B24)*100</f>
@@ -5143,11 +4271,11 @@
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
-        <v>0.0425</v>
+        <v>0.045</v>
       </c>
       <c r="C26" s="29">
         <f>(B26-B25)*100</f>
@@ -5157,11 +4285,11 @@
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
-        <v>0.0425</v>
+        <v>0.045</v>
       </c>
       <c r="C27" s="29">
         <f>(B27-B26)*100</f>
@@ -5171,11 +4299,11 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
-        <v>0.0425</v>
+        <v>0.045</v>
       </c>
       <c r="C28" s="29">
         <f>(B28-B27)*100</f>
@@ -5185,11 +4313,11 @@
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
-        <v>0.0425</v>
+        <v>0.045</v>
       </c>
       <c r="C29" s="29">
         <f>(B29-B28)*100</f>
@@ -5199,7 +4327,7 @@
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -5213,7 +4341,7 @@
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -5227,7 +4355,7 @@
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -5241,7 +4369,7 @@
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -5255,7 +4383,7 @@
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -5269,7 +4397,7 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -5277,6 +4405,90 @@
       </c>
       <c r="C35" s="29">
         <f>(B35-B34)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C36" s="29">
+        <f>(B36-B35)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B37" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C37" s="29">
+        <f>(B37-B36)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C38" s="29">
+        <f>(B38-B37)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C39" s="29">
+        <f>(B39-B38)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C40" s="29">
+        <f>(B40-B39)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="C41" s="29">
+        <f>(B41-B40)*100</f>
         <v/>
       </c>
     </row>
@@ -5316,7 +4528,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5118,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6185,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
@@ -7749,635 +6961,863 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 31/08/2026 01:04</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 31/08/2026 17:52</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de entidad</t>
+          <t>Entidad/tema</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo de fuente</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Analizada en el portal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Banco de Crédito del Perú</t>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Interbank</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Citibank del Perú</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Scotiabank Perú</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>BBVA</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Bancom</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Banco Pichincha</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>BANBIF</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Mibanco</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Banco Falabella</t>
         </is>
       </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Banco Ripley</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Alfin Banco</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Banco Santander</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Banco GNB</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>ICBC Peru bank</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Bank of China(Perú)</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Banco BCI</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Compartamos Banco</t>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Bancos</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Banco Efectiva</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
         </is>
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Financiera QAPAQ</t>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Proempresa</t>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>InFinance XP</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>Financieras</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Financiera Surgir</t>
-        </is>
-      </c>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Arequipa</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Cuzco</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Huancayo</t>
-        </is>
-      </c>
-      <c r="C32" s="30" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B33" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Ica</t>
-        </is>
-      </c>
-      <c r="C33" s="30" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B34" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Maynas</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Del Santa</t>
-        </is>
-      </c>
-      <c r="C35" s="30" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Paita</t>
-        </is>
-      </c>
-      <c r="C36" s="30" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Piura</t>
-        </is>
-      </c>
-      <c r="C37" s="30" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Tacna</t>
-        </is>
-      </c>
-      <c r="C38" s="30" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>CMAC Trujillo</t>
-        </is>
-      </c>
-      <c r="C39" s="30" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>Cajas municipales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Caja Metropolitana</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B41" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Los Andes</t>
-        </is>
-      </c>
-      <c r="C41" s="30" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Prymera</t>
-        </is>
-      </c>
-      <c r="C42" s="30" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Incasur</t>
-        </is>
-      </c>
-      <c r="C43" s="30" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Del Centro</t>
-        </is>
-      </c>
-      <c r="C44" s="30" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Cajas rurales de ahorro y crédito</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>CRAC Cencosud Scotia</t>
-        </is>
-      </c>
-      <c r="C45" s="30" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C45"/>
+  <autoFilter ref="A4:F28"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-09-01 01:36 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -15,14 +15,16 @@
     <sheet name="FSD Y SEGURIDAD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="FICHAS POR ENTIDAD" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TARJETAS DE CREDITO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUENTES Y NOTAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ENTIDADES AUTORIZADAS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUENTES Y NOTAS" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RANKING'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ESCALAS DE TASA'!$A$4:$E$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FICHAS POR ENTIDAD'!$A$4:$L$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TARJETAS DE CREDITO'!$A$4:$J$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ENTIDADES AUTORIZADAS'!$A$4:$C$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FUENTES Y NOTAS'!$A$4:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -180,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -235,6 +237,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -556,12 +561,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'TASA BCRP'!$A$5:$A$41</f>
+              <f>'TASA BCRP'!$A$5:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'TASA BCRP'!$B$5:$B$41</f>
+              <f>'TASA BCRP'!$B$5:$B$40</f>
             </numRef>
           </val>
         </ser>
@@ -1006,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 31/08/2026 17:52. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 01/09/2026 01:36. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1323,873 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 01/09/2026 01:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Entidad/tema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de fuente</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Dato principal</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nivel de confianza</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Video de referencia</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Estructura de pestañas y ranking mostrado</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Alta para diseño; media para vigencia</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Capturas del usuario y video</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>FSD</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>https://fsd.org.pe/</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Cobertura Jun–Ago 2026: S/122,000</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verificar reglas de cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>BCRP</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Tasa de referencia 4.25% a julio de 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Contexto macroeconómico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Guía para comparar productos y leer contratos</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>No es una recomendación de producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Digital – 9.70%</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Financiera SURGIR</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Actualizado frente al video</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Financiera QAPAQ</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Insuperable – 5.00%</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario oficial</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en tarifario de campaña</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Clásico – 5.00%</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Imparable – 4.85%</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tasa verificada; fecha final por confirmar</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Banco Alfin</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Ahorro Meta – 4.80%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Con reserva: verificar vigencia</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Compartamos Financiera</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta WOW – 4.60%</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en campaña oficial</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Tasa y vigencia verificadas; rango por confirmar</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Plus – 4.50%</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Verificar antes de abrir</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Efectiva (Efectibank)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta de Ahorro Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Banco GNB Perú</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Ahorro Rolando – 4.50%</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en web oficial</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Caja Arequipa</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Campaña Caja Digital – 4.50%</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en reglamento oficial</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Caja Piura</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Tasa máxima verificada; umbral reconstruido</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Financiera Oh! / SIP</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Producto / transparencia oficial</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>AhorraMás Soles – 4.00%</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Verificado en fuente oficial</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Reconstrucción columnas I–K</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Inferencia documentada</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>SURGIR</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Diferencia frente al video</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>La tasa actualizada se usa en el ranking y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Vigencia</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>La campaña visible venció 31/07/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Confirmar tarifario desde 01/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Caja Cusco</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>https://www.cmac-cusco.com.pe/</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>No se localizó TyC oficial específico de agosto 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Baja/Media</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F28"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1357,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -2539,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -3354,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -3938,7 +4810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3956,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -3980,22 +4852,22 @@
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>0.0775</v>
+        <v>0.075</v>
       </c>
       <c r="C5" s="24" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>0.075</v>
+        <v>0.0725</v>
       </c>
       <c r="C6" s="29">
         <f>(B6-B5)*100</f>
@@ -4005,11 +4877,11 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>0.0725</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C7" s="29">
         <f>(B7-B6)*100</f>
@@ -4019,11 +4891,11 @@
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.0675</v>
       </c>
       <c r="C8" s="29">
         <f>(B8-B7)*100</f>
@@ -4033,11 +4905,11 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>0.0675</v>
+        <v>0.065</v>
       </c>
       <c r="C9" s="29">
         <f>(B9-B8)*100</f>
@@ -4047,11 +4919,11 @@
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>0.065</v>
+        <v>0.0625</v>
       </c>
       <c r="C10" s="29">
         <f>(B10-B9)*100</f>
@@ -4061,7 +4933,7 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
@@ -4075,11 +4947,11 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>0.0625</v>
+        <v>0.06</v>
       </c>
       <c r="C12" s="29">
         <f>(B12-B11)*100</f>
@@ -4089,11 +4961,11 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>0.06</v>
+        <v>0.0575</v>
       </c>
       <c r="C13" s="29">
         <f>(B13-B12)*100</f>
@@ -4103,7 +4975,7 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
@@ -4117,7 +4989,7 @@
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B15" s="25" t="n">
@@ -4131,11 +5003,11 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>0.0575</v>
+        <v>0.055</v>
       </c>
       <c r="C16" s="29">
         <f>(B16-B15)*100</f>
@@ -4145,11 +5017,11 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
-        <v>0.055</v>
+        <v>0.0525</v>
       </c>
       <c r="C17" s="29">
         <f>(B17-B16)*100</f>
@@ -4159,7 +5031,7 @@
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
@@ -4173,11 +5045,11 @@
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B19" s="25" t="n">
-        <v>0.0525</v>
+        <v>0.05</v>
       </c>
       <c r="C19" s="29">
         <f>(B19-B18)*100</f>
@@ -4187,7 +5059,7 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B20" s="25" t="n">
@@ -4201,11 +5073,11 @@
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B21" s="25" t="n">
-        <v>0.05</v>
+        <v>0.0475</v>
       </c>
       <c r="C21" s="29">
         <f>(B21-B20)*100</f>
@@ -4215,7 +5087,7 @@
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B22" s="25" t="n">
@@ -4229,7 +5101,7 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
@@ -4243,7 +5115,7 @@
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
@@ -4257,11 +5129,11 @@
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B25" s="25" t="n">
-        <v>0.0475</v>
+        <v>0.045</v>
       </c>
       <c r="C25" s="29">
         <f>(B25-B24)*100</f>
@@ -4271,7 +5143,7 @@
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B26" s="25" t="n">
@@ -4285,7 +5157,7 @@
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B27" s="25" t="n">
@@ -4299,7 +5171,7 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
@@ -4313,11 +5185,11 @@
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B29" s="25" t="n">
-        <v>0.045</v>
+        <v>0.0425</v>
       </c>
       <c r="C29" s="29">
         <f>(B29-B28)*100</f>
@@ -4327,7 +5199,7 @@
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="B30" s="25" t="n">
@@ -4341,7 +5213,7 @@
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B31" s="25" t="n">
@@ -4355,7 +5227,7 @@
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B32" s="25" t="n">
@@ -4369,7 +5241,7 @@
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B33" s="25" t="n">
@@ -4383,7 +5255,7 @@
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B34" s="25" t="n">
@@ -4397,7 +5269,7 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B35" s="25" t="n">
@@ -4411,7 +5283,7 @@
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B36" s="25" t="n">
@@ -4425,7 +5297,7 @@
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B37" s="25" t="n">
@@ -4439,7 +5311,7 @@
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B38" s="25" t="n">
@@ -4453,7 +5325,7 @@
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B39" s="25" t="n">
@@ -4467,7 +5339,7 @@
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B40" s="25" t="n">
@@ -4475,20 +5347,6 @@
       </c>
       <c r="C40" s="29">
         <f>(B40-B39)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="C41" s="29">
-        <f>(B41-B40)*100</f>
         <v/>
       </c>
     </row>
@@ -4528,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -6185,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
@@ -6961,863 +7819,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FUENTES, ALCANCES Y LIMITACIONES</t>
+          <t>ENTIDADES AUTORIZADAS A CAPTAR DEPOSITOS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 31/08/2026 17:52</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 01/09/2026 01:36</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Entidad/tema</t>
+          <t>Tipo de entidad</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tipo de fuente</t>
+          <t>Entidad</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Dato principal</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Nivel de confianza</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Video de referencia</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>YouTube</t>
+          <t>Analizada en el portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Banco de Crédito del Perú</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Estructura de pestañas y ranking mostrado</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Alta para diseño; media para vigencia</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Capturas del usuario y video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>FSD</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>https://fsd.org.pe/</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cobertura Jun–Ago 2026: S/122,000</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Verificar reglas de cobertura</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>BCRP</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Tasa de referencia 4.25% a julio de 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Contexto macroeconómico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>SBS</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Oficial</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Interbank</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Citibank del Perú</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Scotiabank Perú</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>https://www.sbs.gob.pe/usuarios/aprende-con-la-sbs/compara-y-elige</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Guía para comparar productos y leer contratos</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>No es una recomendación de producto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Scotiabank Perú</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>https://www.scotiabank.com.pe/Personas/Ahorros/Cuentas-Bancarias/cuenta-digital</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Digital – 9.70%</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>La TREA promocional no se aplica a todo el saldo: máximo remunerado S/3,000; el exceso recibe la tasa regular indicada por el banco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Financiera SURGIR</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>https://www.surgir.com.pe/tasas-y-tarifas</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Gold Select – 5.60%</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Actualizado frente al video</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia relevante: el video muestra 5.25%, mientras la página oficial consultada publica hasta 5.60%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Bancom</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Banco Pichincha</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>BANBIF</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Mibanco</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Banco Falabella</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Banco Ripley</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Alfin Banco</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Banco Santander</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Banco GNB</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ICBC Peru bank</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Bank of China(Perú)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Banco BCI</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Santander Consumer Bank</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Compartamos Banco</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Banco Efectiva</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Confianza</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Financiera QAPAQ</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>https://www.qapaq.pe/wp-content/uploads/2025/04/Tarifario-ahorros-Insuperable-Abril-2025.pdf</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Insuperable – 5.00%</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario oficial</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>La versión digital puede no exigir monto mínimo de apertura. La tasa depende del saldo; no basta con abrir la cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Confianza</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>https://confianza.pe/docs/2026/07/T008-027%20Tarifario%20Campana%20-%20Ahorro%20Comun%20en%20Canal%20Digital.pdf</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Común – canal digital – 5.00%</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en tarifario de campaña</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>La tasa promocional depende del canal digital y del rango de saldo establecido en el tarifario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Banco Falabella</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancofalabella.pe/promociones/detalle/tasa-preferencial-cuenta-sueldo</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Clásico – 5.00%</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>La tasa regular publicada para la Cuenta Ahorro Clásico es menor; el 5% exige abono de sueldo y tiene tope de saldo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Santander Consumer Bank</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>https://www.santanderconsumer.com.pe/wp-content/uploads/2026/07/TERMINOS-Y-CONDICIONES-WEB-LA-JUGADA-DEL-AHORRO-1.pdf</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Imparable – 4.85%</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Tasa verificada; fecha final por confirmar</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>El documento enlazado corresponde a una campaña complementaria; revisar también cartilla y tarifario antes de contratar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Banco Alfin</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>https://www.alfinbanco.pe/ahorros/ahorrometa</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Ahorro Meta – 4.80%</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>La tasa depende del canal de apertura. El simulador usa 4.80% como escenario web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/api/storage/file/Qo95UD7M0bMGuYblDSEeD8CMd2xkUkBoXlRGADLQ.pdf</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta digital Wayki / campaña Ahorra y Gana – 4.75%</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Con reserva: verificar vigencia</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>El PDF enlazado es una campaña oficial anterior localizada como referencia. No debe asumirse que sus condiciones siguen vigentes en agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Compartamos Financiera</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="inlineStr">
-        <is>
-          <t>https://www.compartamos.com.pe/wcm/connect/a5b7bede-8d6a-4eb1-923f-084d0d3928f7/Camp_Cuenta_Wow.pdf?MOD=AJPERES</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta WOW – 4.60%</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en campaña oficial</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>El ITF aplicable es 0.005%, conforme a la regulación y condiciones informadas por la entidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancom.pe/personas/promociones/cuenta-ahorro</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorros Soles – promoción digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Tasa y vigencia verificadas; rango por confirmar</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Esta entidad se incorporó como mejor reconstrucción de una de las columnas ocultas I–K del video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Plus – 4.50%</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Verificar antes de abrir</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Se mantiene en el comparativo porque aparece en el video, pero la tasa debe confirmarse en el tarifario vigente de agosto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Efectiva (Efectibank)</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr">
-        <is>
-          <t>https://www.efectiva.com.pe/ahorros/cuenta-de-ahorros/</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de Ahorro Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>La web del producto enlaza contrato multiproducto, cartilla, tarifario y fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Banco GNB Perú</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t>https://www.bancognb.com.pe/inicio/banca-personas/cuentas/cuenta-rolando</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Ahorro Rolando – 4.50%</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en web oficial</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>La capitalización diaria es una característica diferenciadora; el simulador anualiza mediante TREA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>Caja Arequipa</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajaarequipa.pe/wp-content/uploads/2026/07/Reglamento-campana-digital-vigente-desde-24-julio-set.2026-caja-digital.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Campaña Caja Digital – 4.50%</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en reglamento oficial</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>La apertura debe realizarse por los canales digitales autorizados; no aplica a aperturas en agencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>Caja Piura</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cajapiura.pe/campaigns-sweepstakes/details/gana-mas-con-cuenta-light</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta Light – Ahorra y gana más – 4.50%</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Tasa máxima verificada; umbral reconstruido</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>La web oficial publica 'hasta 4.5%' y apertura desde S/100; el rango exacto de la tasa máxima debe revisarse en TyC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Financiera Oh! / SIP</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Producto / transparencia oficial</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>https://cms.sip.pe/wp-content/documentos/ahorra-mas/Cartilla-AhorraMas-Ahorros.pdf</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>AhorraMás Soles – 4.00%</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Verificado en fuente oficial</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>El contrato contempla cierre automático en determinadas circunstancias de inactividad; revisar cláusulas completas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Reconstrucción columnas I–K</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Inferencia documentada</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=rFvo7DurR8M</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco, Compartamos y Banco de Comercio</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Las tres columnas no aparecen en las capturas adjuntas; se eligieron por consistencia con el orden de tasas y campañas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SURGIR</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Diferencia frente al video</t>
-        </is>
-      </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>https://www.surgir.com.pe/cuenta-gold-select</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Web oficial: hasta 5.60%; video: 5.25%</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>La tasa actualizada se usa en el ranking y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Banco Ripley</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Vigencia</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Proempresa</t>
         </is>
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>https://www.bancoripley.com.pe/ahorros/cuenta-ahorros.html</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>La campaña visible venció 31/07/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Confirmar tarifario desde 01/08/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Caja Cusco</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Limitación</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>https://www.cmac-cusco.com.pe/</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>No se localizó TyC oficial específico de agosto 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Baja/Media</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>La tasa de 4.75% se conserva como reconstrucción del video y se marca con reserva.</t>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>InFinance XP</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Financiera Surgir</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Arequipa</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Cuzco</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Huancayo</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Ica</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Maynas</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Del Santa</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Paita</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Piura</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Tacna</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>CMAC Trujillo</t>
+        </is>
+      </c>
+      <c r="C39" s="30" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Cajas municipales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t>Caja Metropolitana</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Los Andes</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Prymera</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Incasur</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Del Centro</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Cajas rurales de ahorro y crédito</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>CRAC Cencosud Scotia</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="inlineStr">
+        <is>
+          <t>Miembros del Fondo de Seguro de Depositos, administrado por la SBS. Equivale a las empresas autorizadas a captar depositos del publico. Las cooperativas (COOPAC) no son miembros del FSD: cuentan con un fondo propio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F28"/>
+  <autoFilter ref="A4:C45"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-09-01 15:22 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 01/09/2026 01:36. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 01/09/2026 15:22. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 01/09/2026 01:36</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 01/09/2026 15:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-09-02 00:47 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 01/09/2026 15:22. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 02/09/2026 00:47. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 01/09/2026 15:22</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 02/09/2026 00:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: actualizacion automatica 2026-09-02 14:56 UTC
</commit_message>
<xml_diff>
--- a/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
+++ b/docs/descargas/Ranking_Cuentas_Ahorro_Peru_Agosto_2026_MEJORADO.xlsx
@@ -1011,7 +1011,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corte de datos: 2026-08-06   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Corte de datos: 2026-08-06   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Libro generado el 02/09/2026 00:47. La fecha de tu descarga va en el nombre del archivo.</t>
+          <t>Libro generado el 02/09/2026 14:56. La fecha de tu descarga va en el nombre del archivo.</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Registro de fuentes oficiales y campos que requieren confirmacion directa.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Ordenado por TREA descendente. Corte: 2026-08-06. Cifras en formato numerico corregido. No constituye recomendacion financiera.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Tramos consolidados de las 16 entidades. En el original estaban dispersos en cada hoja.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Edita el monto (B5) y el plazo (B6). Las formulas recalculan solas. TREA efectiva anual con capitalizacion mensual.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Serie mensual PD04722MM. Vigente: 4.25%. Fuente: https://estadisticas.bcrp.gob.pe/estadisticas/series/mensuales/resultados/PD04722MM/html   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Cobertura vigente: S/122,000 por depositante y por institucion. Fuente: https://fsd.org.pe/   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Todos los campos de las 16 hojas individuales del original, en una sola tabla filtrable.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Ordenadas por TCEA ascendente: aqui gana la tasa MAS BAJA. Cifras referenciales.   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 02/09/2026 00:47</t>
+          <t>Miembros del Fondo de Seguro de Depositos (administrado por la SBS). Total: 41. Fuente: https://fsd.org.pe/miembros/   ·   Datos generados el 02/09/2026 14:56</t>
         </is>
       </c>
     </row>

</xml_diff>